<commit_message>
Sync BD docs 2026-07-06-v3 (202607060338) from my-cloud-project@6a66d5a
</commit_message>
<xml_diff>
--- a/Grim_Pillars_Oracle_BD指南.xlsx
+++ b/Grim_Pillars_Oracle_BD指南.xlsx
@@ -1959,7 +1959,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>版本 2026-07-06-v2 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充</t>
+          <t>版本 2026-07-06-v3 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>版本 2026-07-06-v2 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充</t>
+          <t>版本 2026-07-06-v3 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>版本 2026-07-06-v2 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充 · 02-技能请向右滚动至 I 列</t>
+          <t>版本 2026-07-06-v3 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充 · 02-技能请向右滚动至 I 列</t>
         </is>
       </c>
     </row>
@@ -4486,7 +4486,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>版本 2026-07-06-v2 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充</t>
+          <t>版本 2026-07-06-v3 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充</t>
         </is>
       </c>
     </row>
@@ -5879,7 +5879,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>版本 2026-07-06-v2 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充</t>
+          <t>版本 2026-07-06-v3 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>常见问题 · 2026-07-06-v2</t>
+          <t>常见问题 · 2026-07-06-v3</t>
         </is>
       </c>
     </row>
@@ -7434,7 +7434,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>版本 2026-07-06-v2 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充 · 汇总页；各表右侧绿底列为可编辑 FAQ</t>
+          <t>版本 2026-07-06-v3 · 各表表格最右列为【常见问题】（浅绿底），可直接编辑补充 · 汇总页；各表右侧绿底列为可编辑 FAQ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607130115) from my-cloud-project@aba4965
</commit_message>
<xml_diff>
--- a/Grim_Pillars_Oracle_BD指南.xlsx
+++ b/Grim_Pillars_Oracle_BD指南.xlsx
@@ -1393,7 +1393,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6477000" cy="3895725"/>
+    <ext cx="6019800" cy="4476750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1415,7 +1415,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>101</row>
+      <row>105</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -1907,14 +1907,14 @@
     <row r="5" outlineLevel="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>参考数据：Runes of Aldur · Lv.98 Oracle（poe.ninja 面板快照）</t>
+          <t>参考数据：Runes of Aldur · Lv.99 Oracle（poe.ninja 面板快照）</t>
         </is>
       </c>
     </row>
     <row r="6" outlineLevel="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>数据更新：2026-07-07 · PoE2 0.5.4</t>
+          <t>数据更新：2026-07-12 · PoE2 0.5.4</t>
         </is>
       </c>
     </row>
@@ -4386,7 +4386,7 @@
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>68（I组面板）</t>
+          <t>63（I组面板）</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>248</t>
+          <t>253</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>6,767</t>
+          <t>6,713</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Str 仅 68+6，只能选低需求盾底</t>
+          <t>Str 仅 63+6，只能选低需求盾底</t>
         </is>
       </c>
     </row>
@@ -4817,7 +4817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4852,7 +4852,7 @@
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>图例：蓝 = 升华轮盘 · 浅蓝 = 未见之道 · 红 = 基石 · 黄 = notable · 灰 = 普通小点
-已点节点数：112（来源 poe.ninja passiveSelection）</t>
+已点节点数：114（来源 poe.ninja passiveSelection）</t>
         </is>
       </c>
     </row>
@@ -4885,178 +4885,94 @@
     <row r="32" outlineLevel="1"/>
     <row r="33" outlineLevel="1"/>
     <row r="34" outlineLevel="1"/>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>▸ 职业与升华</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" outlineLevel="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>项目</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>内容</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" outlineLevel="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>基础职业</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>德鲁伊（Druid）</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>角色底层职业</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" outlineLevel="1">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>使用升华</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>天启先知（Oracle）</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>升华试炼选择</t>
-        </is>
-      </c>
-    </row>
+    <row r="35" outlineLevel="1"/>
+    <row r="36" outlineLevel="1"/>
+    <row r="37" outlineLevel="1"/>
+    <row r="38" outlineLevel="1"/>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>▸ 基石与核心天赋</t>
+          <t>▸ 职业与升华</t>
         </is>
       </c>
     </row>
     <row r="40" outlineLevel="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>类型</t>
+          <t>项目</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>名称</t>
+          <t>内容</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>作用</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>备注</t>
+          <t>说明</t>
         </is>
       </c>
     </row>
     <row r="41" outlineLevel="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>基石</t>
+          <t>基础职业</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Pain Attunement</t>
+          <t>德鲁伊（Druid）</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>已点</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>角色底层职业</t>
         </is>
       </c>
     </row>
     <row r="42" outlineLevel="1">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>基石</t>
+          <t>使用升华</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Ancestral Bond</t>
+          <t>天启先知（Oracle）</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>已点</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" outlineLevel="1">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>基石</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>Mind Over Matter</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>已点</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>升华试炼选择</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>▸ 基石与核心天赋</t>
         </is>
       </c>
     </row>
     <row r="44" outlineLevel="1">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>基石</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>Scarred Faith</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>已点</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>作用</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>备注</t>
         </is>
       </c>
     </row>
@@ -5068,7 +4984,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Elemental Equilibrium</t>
+          <t>Pain Attunement</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -5090,7 +5006,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Wildsurge Incantation</t>
+          <t>Ancestral Bond</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -5107,230 +5023,210 @@
     <row r="47" outlineLevel="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>涂油</t>
+          <t>基石</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Warding Fetish</t>
+          <t>Mind Over Matter</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>每诅咒 +30% 伤害，-30% 诅咒效果</t>
+          <t>已点</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>核心</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="48" outlineLevel="1">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>武器组 I</t>
+          <t>基石</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>24 点</t>
+          <t>Scarred Faith</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>冰霜/法术/暴击/图腾伤害</t>
+          <t>已点</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>输出专精</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="49" outlineLevel="1">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>武器组 II</t>
+          <t>基石</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>24 点</t>
+          <t>Elemental Equilibrium</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>护甲/抗性/法力/格挡</t>
+          <t>已点</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>生存专精</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>▸ 升华试炼天赋（8 点 · 天启先知轮盘）</t>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" outlineLevel="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>基石</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Wildsurge Incantation</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>已点</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="51" outlineLevel="1">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>序号</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>天赋</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>效果</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>类型</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>校验</t>
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>涂油</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Warding Fetish</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>每诅咒 +30% 伤害，-30% 诅咒效果</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>核心</t>
         </is>
       </c>
     </row>
     <row r="52" outlineLevel="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>武器组 I</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>虛實交織</t>
+          <t>24 点</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>已配置基石中型范围内未连接的非基石天赋仍可配置</t>
+          <t>冰霜/法术/暴击/图腾伤害</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>升华核心</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
+          <t>输出专精</t>
         </is>
       </c>
     </row>
     <row r="53" outlineLevel="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>武器组 II</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>未見之道</t>
+          <t>24 点</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>踏上未履之道；解锁先知专属天赋树分支</t>
+          <t>护甲/抗性/法力/格挡</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>升华核心</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" outlineLevel="1">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>無名心木</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>+1 召唤图腾上限；图腾生命归零后 6 秒死亡</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>升华核心</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
+          <t>生存专精</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>▸ 升华试炼天赋（8 点 · 天启先知轮盘）</t>
         </is>
       </c>
     </row>
     <row r="55" outlineLevel="1">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>微小損害</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>敌人对你暴击率不幸；敌人击中你伤害不幸</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>升华核心</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>天赋</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>效果</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>校验</t>
         </is>
       </c>
     </row>
     <row r="56" outlineLevel="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>天赋点</t>
+          <t>虛實交織</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>获得 1 点天赋点</t>
+          <t>已配置基石中型范围内未连接的非基石天赋仍可配置</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>升华小点</t>
+          <t>升华核心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -5342,22 +5238,22 @@
     <row r="57" outlineLevel="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>天赋点</t>
+          <t>未見之道</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>获得 1 点天赋点</t>
+          <t>踏上未履之道；解锁先知专属天赋树分支</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>升华小点</t>
+          <t>升华核心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -5369,22 +5265,22 @@
     <row r="58" outlineLevel="1">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>對你的暴擊傷害加成</t>
+          <t>無名心木</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>击中你的伤害减少 12% 暴击伤害加成</t>
+          <t>+1 召唤图腾上限；图腾生命归零后 6 秒死亡</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>升华小点</t>
+          <t>升华核心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -5396,83 +5292,103 @@
     <row r="59" outlineLevel="1">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>圖騰攻擊及施放速度</t>
+          <t>微小損害</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>图腾法术施放速度 +5%；图腾攻击速度 +5%</t>
+          <t>敌人对你暴击率不幸；敌人击中你伤害不幸</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
+          <t>升华核心</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" outlineLevel="1">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>天赋点</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>获得 1 点天赋点</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>✓poe2db</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>▸ 未见之道天赋（8 点 · 需先点「未见之道」）</t>
-        </is>
-      </c>
-    </row>
     <row r="61" outlineLevel="1">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>序号</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>天赋</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>效果</t>
-        </is>
-      </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>类型</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>校验</t>
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>天赋点</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>获得 1 点天赋点</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>升华小点</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
         </is>
       </c>
     </row>
     <row r="62" outlineLevel="1">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>精算獵者</t>
+          <t>對你的暴擊傷害加成</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>减少 5% 技能速度；提高 50% 暴击率</t>
+          <t>击中你的伤害减少 12% 暴击伤害加成</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>升华核心</t>
+          <t>升华小点</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -5484,22 +5400,22 @@
     <row r="63" outlineLevel="1">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>同袍情誼</t>
+          <t>圖騰攻擊及施放速度</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>提高 30% 伤害；召唤物造成 30% 更多伤害</t>
+          <t>图腾法术施放速度 +5%；图腾攻击速度 +5%</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>升华核心</t>
+          <t>升华小点</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -5508,79 +5424,59 @@
         </is>
       </c>
     </row>
-    <row r="64" outlineLevel="1">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="inlineStr">
-        <is>
-          <t>暴擊傷害</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>提高 20% 暴击伤害加成</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>升华小点</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>▸ 未见之道天赋（8 点 · 需先点「未见之道」）</t>
         </is>
       </c>
     </row>
     <row r="65" outlineLevel="1">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>暴擊傷害</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>提高 20% 暴击伤害加成</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>升华小点</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>天赋</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>效果</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>校验</t>
         </is>
       </c>
     </row>
     <row r="66" outlineLevel="1">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>暴擊傷害</t>
+          <t>精算獵者</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>提高 20% 暴击伤害加成</t>
+          <t>减少 5% 技能速度；提高 50% 暴击率</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>升华小点</t>
+          <t>升华核心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -5592,22 +5488,22 @@
     <row r="67" outlineLevel="1">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>傷害和召喚物傷害</t>
+          <t>同袍情誼</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>提高 15% 伤害；召唤物造成 15% 更多伤害</t>
+          <t>提高 30% 伤害；召唤物造成 30% 更多伤害</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>升华小点</t>
+          <t>升华核心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -5619,17 +5515,17 @@
     <row r="68" outlineLevel="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>傷害和召喚物傷害</t>
+          <t>暴擊傷害</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>提高 15% 伤害；召唤物造成 15% 更多伤害</t>
+          <t>提高 20% 暴击伤害加成</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
@@ -5646,585 +5542,693 @@
     <row r="69" outlineLevel="1">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
+          <t>暴擊傷害</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>提高 20% 暴击伤害加成</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>升华小点</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" outlineLevel="1">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>暴擊傷害</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>提高 20% 暴击伤害加成</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>升华小点</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" outlineLevel="1">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
           <t>傷害和召喚物傷害</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr">
+      <c r="C71" s="5" t="inlineStr">
         <is>
           <t>提高 15% 伤害；召唤物造成 15% 更多伤害</t>
         </is>
       </c>
-      <c r="D69" s="5" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E69" s="5" t="inlineStr">
+      <c r="E71" s="5" t="inlineStr">
         <is>
           <t>✓poe2db</t>
         </is>
       </c>
     </row>
-    <row r="70" outlineLevel="1">
-      <c r="A70" s="6" t="inlineStr">
-        <is>
-          <t>升华数据已与 poe2db.tw 交叉验证（16/16 条）</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>▸ 武器组 I 天赋要点（24 点 · 伤害）</t>
-        </is>
-      </c>
-    </row>
     <row r="72" outlineLevel="1">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>方向</t>
-        </is>
-      </c>
-      <c r="B72" s="4" t="inlineStr">
-        <is>
-          <t>优先词缀类</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>备注</t>
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>傷害和召喚物傷害</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>提高 15% 伤害；召唤物造成 15% 更多伤害</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>升华小点</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
         </is>
       </c>
     </row>
     <row r="73" outlineLevel="1">
       <c r="A73" s="5" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>傷害和召喚物傷害</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>提高 15% 伤害；召唤物造成 15% 更多伤害</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>升华小点</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" outlineLevel="1">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>升华数据已与 poe2db.tw 交叉验证（16/16 条）</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>▸ 武器组 I 天赋要点（24 点 · 伤害）</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" outlineLevel="1">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>方向</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>优先词缀类</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" outlineLevel="1">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
           <t>伤害</t>
         </is>
       </c>
-      <c r="B73" s="5" t="inlineStr">
+      <c r="B77" s="5" t="inlineStr">
         <is>
           <t>冰霜 / 法术 / 暴击 / 图腾伤害</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
+      <c r="C77" s="5" t="inlineStr">
         <is>
           <t>Grim Pillars 主输出</t>
         </is>
       </c>
     </row>
-    <row r="74" outlineLevel="1">
-      <c r="A74" s="5" t="inlineStr">
+    <row r="78" outlineLevel="1">
+      <c r="A78" s="5" t="inlineStr">
         <is>
           <t>图腾</t>
         </is>
       </c>
-      <c r="B74" s="5" t="inlineStr">
+      <c r="B78" s="5" t="inlineStr">
         <is>
           <t>图腾数量、施放速度、生命</t>
         </is>
       </c>
-      <c r="C74" s="5" t="inlineStr">
+      <c r="C78" s="5" t="inlineStr">
         <is>
           <t>配合 Ancestral Bond + Heartwood</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" outlineLevel="1">
-      <c r="A75" s="5" t="inlineStr">
-        <is>
-          <t>诅咒</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="inlineStr">
-        <is>
-          <t>诅咒效果、额外诅咒槽</t>
-        </is>
-      </c>
-      <c r="C75" s="5" t="inlineStr">
-        <is>
-          <t>Blasphemy 链路</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" outlineLevel="1">
-      <c r="A76" s="5" t="inlineStr">
-        <is>
-          <t>法力</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>最大法力、回复、Archmage 协同</t>
-        </is>
-      </c>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>MoM + EB 第二血条</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="3" t="inlineStr">
-        <is>
-          <t>▸ 武器组 II 天赋要点（24 点 · 防御）</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" outlineLevel="1">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <t>方向</t>
-        </is>
-      </c>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t>优先词缀类</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>备注</t>
         </is>
       </c>
     </row>
     <row r="79" outlineLevel="1">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>护甲</t>
+          <t>诅咒</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>护甲%、元素承伤转护甲</t>
+          <t>诅咒效果、额外诅咒槽</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>物承伤尖刺时切换</t>
+          <t>Blasphemy 链路</t>
         </is>
       </c>
     </row>
     <row r="80" outlineLevel="1">
       <c r="A80" s="5" t="inlineStr">
         <is>
+          <t>法力</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>最大法力、回复、Archmage 协同</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>MoM + EB 第二血条</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>▸ 武器组 II 天赋要点（24 点 · 防御）</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" outlineLevel="1">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>方向</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>优先词缀类</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" outlineLevel="1">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>护甲</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>护甲%、元素承伤转护甲</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>物承伤尖刺时切换</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" outlineLevel="1">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
           <t>抗性</t>
         </is>
       </c>
-      <c r="B80" s="5" t="inlineStr">
+      <c r="B84" s="5" t="inlineStr">
         <is>
           <t>全抗 / 闪电抗补满</t>
         </is>
       </c>
-      <c r="C80" s="5" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr">
         <is>
           <t>配合 Eternal Spark +30%</t>
         </is>
       </c>
     </row>
-    <row r="81" outlineLevel="1">
-      <c r="A81" s="5" t="inlineStr">
+    <row r="85" outlineLevel="1">
+      <c r="A85" s="5" t="inlineStr">
         <is>
           <t>格挡</t>
         </is>
       </c>
-      <c r="B81" s="5" t="inlineStr">
+      <c r="B85" s="5" t="inlineStr">
         <is>
           <t>格挡率与格挡效果</t>
         </is>
       </c>
-      <c r="C81" s="5" t="inlineStr">
+      <c r="C85" s="5" t="inlineStr">
         <is>
           <t>当前 0%，可选投资</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" outlineLevel="1">
-      <c r="A82" s="5" t="inlineStr">
-        <is>
-          <t>法力</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>保留与 Spirit 相关</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>双勾技能不灰</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="3" t="inlineStr">
-        <is>
-          <t>▸ 加点顺序（待补充 · 占位模板）</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" outlineLevel="1">
-      <c r="A84" s="6" t="inlineStr">
-        <is>
-          <t>后续可按 PoB 导出或开荒录像填写具体节点名称与顺序。</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" outlineLevel="1">
-      <c r="A85" s="4" t="inlineStr">
-        <is>
-          <t>优先级</t>
-        </is>
-      </c>
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>阶段</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>天赋/节点</t>
-        </is>
-      </c>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>说明</t>
         </is>
       </c>
     </row>
     <row r="86" outlineLevel="1">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>法力</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>开荒</t>
+          <t>保留与 Spirit 相关</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>（待填）图腾 / 法术基础小点</t>
-        </is>
-      </c>
-      <c r="D86" s="5" t="inlineStr">
-        <is>
-          <t>Act 1–2 清图与 Boss</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" outlineLevel="1">
-      <c r="A87" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="inlineStr">
-        <is>
-          <t>中期</t>
-        </is>
-      </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>（待填）Spell Totem + 诅咒链路</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
-        <is>
-          <t>Bone Cage → Grim Pillars 转折</t>
+          <t>双勾技能不灰</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>▸ 加点顺序（待补充 · 占位模板）</t>
         </is>
       </c>
     </row>
     <row r="88" outlineLevel="1">
-      <c r="A88" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B88" s="5" t="inlineStr">
-        <is>
-          <t>成型</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>（待填）MoM / EB / Archmage 路径</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>法力池与低血 PA</t>
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>后续可按 PoB 导出或开荒录像填写具体节点名称与顺序。</t>
         </is>
       </c>
     </row>
     <row r="89" outlineLevel="1">
-      <c r="A89" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="inlineStr">
-        <is>
-          <t>升华</t>
-        </is>
-      </c>
-      <c r="C89" s="5" t="inlineStr">
-        <is>
-          <t>（待填）轮盘 8 点顺序</t>
-        </is>
-      </c>
-      <c r="D89" s="5" t="inlineStr">
-        <is>
-          <t>Entwined → Unseen Path → Heartwood…</t>
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>阶段</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>天赋/节点</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>说明</t>
         </is>
       </c>
     </row>
     <row r="90" outlineLevel="1">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>毕业</t>
+          <t>开荒</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>（待填）未见之道 8 点</t>
+          <t>（待填）图腾 / 法术基础小点</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>暴击 / 伤害小点收尾</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="3" t="inlineStr">
-        <is>
-          <t>▸ 过渡计划（待补充 · 占位模板）</t>
+          <t>Act 1–2 清图与 Boss</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" outlineLevel="1">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>中期</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>（待填）Spell Totem + 诅咒链路</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Bone Cage → Grim Pillars 转折</t>
         </is>
       </c>
     </row>
     <row r="92" outlineLevel="1">
-      <c r="A92" s="6" t="inlineStr">
-        <is>
-          <t>记录等级里程碑、天赋重洗与装备更换节点，便于复刻开荒路线。</t>
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>成型</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>（待填）MoM / EB / Archmage 路径</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>法力池与低血 PA</t>
         </is>
       </c>
     </row>
     <row r="93" outlineLevel="1">
-      <c r="A93" s="4" t="inlineStr">
-        <is>
-          <t>里程碑</t>
-        </is>
-      </c>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>等级</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>天赋变化</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>装备变化</t>
-        </is>
-      </c>
-      <c r="E93" s="4" t="inlineStr">
-        <is>
-          <t>备注</t>
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>升华</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>（待填）轮盘 8 点顺序</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>Entwined → Unseen Path → Heartwood…</t>
         </is>
       </c>
     </row>
     <row r="94" outlineLevel="1">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>Lv.28 前</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>毕业</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>（待填）</t>
+          <t>（待填）未见之道 8 点</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>（待填）</t>
-        </is>
-      </c>
-      <c r="E94" s="5" t="inlineStr">
-        <is>
-          <t>基础图腾开荒</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" outlineLevel="1">
-      <c r="A95" s="5" t="inlineStr">
-        <is>
-          <t>Lv.45</t>
-        </is>
-      </c>
-      <c r="B95" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C95" s="5" t="inlineStr">
-        <is>
-          <t>（待填）</t>
-        </is>
-      </c>
-      <c r="D95" s="5" t="inlineStr">
-        <is>
-          <t>（待填）</t>
-        </is>
-      </c>
-      <c r="E95" s="5" t="inlineStr">
-        <is>
-          <t>诅咒 + 低血过渡</t>
+          <t>暴击 / 伤害小点收尾</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>▸ 过渡计划（待补充 · 占位模板）</t>
         </is>
       </c>
     </row>
     <row r="96" outlineLevel="1">
-      <c r="A96" s="5" t="inlineStr">
-        <is>
-          <t>Lv.65</t>
-        </is>
-      </c>
-      <c r="B96" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>（待填）</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="inlineStr">
-        <is>
-          <t>Soul Mantle 入手</t>
-        </is>
-      </c>
-      <c r="E96" s="5" t="inlineStr">
-        <is>
-          <t>自诅咒伤害链启动</t>
+      <c r="A96" s="6" t="inlineStr">
+        <is>
+          <t>记录等级里程碑、天赋重洗与装备更换节点，便于复刻开荒路线。</t>
         </is>
       </c>
     </row>
     <row r="97" outlineLevel="1">
-      <c r="A97" s="5" t="inlineStr">
-        <is>
-          <t>Lv.80+</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>（待填）</t>
-        </is>
-      </c>
-      <c r="D97" s="5" t="inlineStr">
-        <is>
-          <t>II 组装备就位</t>
-        </is>
-      </c>
-      <c r="E97" s="5" t="inlineStr">
-        <is>
-          <t>洗 24 点防御专精</t>
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>等级</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>天赋变化</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>装备变化</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>备注</t>
         </is>
       </c>
     </row>
     <row r="98" outlineLevel="1">
       <c r="A98" s="5" t="inlineStr">
         <is>
+          <t>Lv.28 前</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>（待填）</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>（待填）</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>基础图腾开荒</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" outlineLevel="1">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>Lv.45</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>（待填）</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>（待填）</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>诅咒 + 低血过渡</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" outlineLevel="1">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>Lv.65</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>（待填）</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>Soul Mantle 入手</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>自诅咒伤害链启动</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" outlineLevel="1">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>Lv.80+</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>（待填）</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>II 组装备就位</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>洗 24 点防御专精</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" outlineLevel="1">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
           <t>毕业</t>
         </is>
       </c>
-      <c r="B98" s="5" t="inlineStr">
+      <c r="B102" s="5" t="inlineStr">
         <is>
           <t>98</t>
         </is>
       </c>
-      <c r="C98" s="5" t="inlineStr">
+      <c r="C102" s="5" t="inlineStr">
         <is>
           <t>（待填）</t>
         </is>
       </c>
-      <c r="D98" s="5" t="inlineStr">
+      <c r="D102" s="5" t="inlineStr">
         <is>
           <t>全暗金 + 涂油</t>
         </is>
       </c>
-      <c r="E98" s="5" t="inlineStr">
+      <c r="E102" s="5" t="inlineStr">
         <is>
           <t>对照 ninja 快照微调</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="3" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
         <is>
           <t>▸ Warding Fetish 涂油（贴图）</t>
         </is>
       </c>
     </row>
-    <row r="100" outlineLevel="1">
-      <c r="A100" s="4" t="inlineStr">
+    <row r="104" outlineLevel="1">
+      <c r="A104" s="4" t="inlineStr">
         <is>
           <t>部位</t>
         </is>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B104" s="4" t="inlineStr">
         <is>
           <t>贴图</t>
         </is>
       </c>
-      <c r="C100" s="4" t="inlineStr">
+      <c r="C104" s="4" t="inlineStr">
         <is>
           <t>装备词条</t>
         </is>
       </c>
     </row>
-    <row r="101" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A101" s="10" t="inlineStr">
+    <row r="105" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A105" s="10" t="inlineStr">
         <is>
           <t>涂油</t>
         </is>
       </c>
-      <c r="B101" s="14" t="inlineStr">
+      <c r="B105" s="14" t="inlineStr">
         <is>
           <t>守護神器
 (Warding Fetish)</t>
         </is>
       </c>
-      <c r="C101" s="15" t="n"/>
-    </row>
-    <row r="102" outlineLevel="1" ht="132" customHeight="1">
-      <c r="A102" s="12" t="n"/>
-      <c r="B102" s="13" t="inlineStr"/>
-      <c r="C102" s="5" t="inlineStr">
+      <c r="C105" s="15" t="n"/>
+    </row>
+    <row r="106" outlineLevel="1" ht="132" customHeight="1">
+      <c r="A106" s="12" t="n"/>
+      <c r="B106" s="13" t="inlineStr"/>
+      <c r="C106" s="5" t="inlineStr">
         <is>
           <t>守護神器 (Warding Fetish)
 ■ 你身上每有一個詛咒，增加30%傷害
@@ -6236,27 +6240,27 @@
         </is>
       </c>
     </row>
-    <row r="103" outlineLevel="1"/>
+    <row r="107" outlineLevel="1"/>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A71:F71"/>
-    <mergeCell ref="A99:F99"/>
-    <mergeCell ref="A60:F60"/>
-    <mergeCell ref="A84:F84"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="B105:C105"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A70:F70"/>
-    <mergeCell ref="A91:F91"/>
-    <mergeCell ref="A77:F77"/>
-    <mergeCell ref="B101:C101"/>
-    <mergeCell ref="A83:F83"/>
-    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A75:F75"/>
+    <mergeCell ref="A81:F81"/>
+    <mergeCell ref="A95:F95"/>
+    <mergeCell ref="A103:F103"/>
+    <mergeCell ref="A74:F74"/>
+    <mergeCell ref="A88:F88"/>
+    <mergeCell ref="A105:A106"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="A92:F92"/>
+    <mergeCell ref="A87:F87"/>
+    <mergeCell ref="A96:F96"/>
     <mergeCell ref="A39:F39"/>
-    <mergeCell ref="A101:A102"/>
+    <mergeCell ref="A64:F64"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6317,7 +6321,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Grim Pillars 414,709</t>
+          <t>Grim Pillars 436,868</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607160420) from my-cloud-project@d551727
</commit_message>
<xml_diff>
--- a/Grim_Pillars_Oracle_BD指南.xlsx
+++ b/Grim_Pillars_Oracle_BD指南.xlsx
@@ -5216,7 +5216,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>虚实交织</t>
+          <t>虛實交織</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -5229,7 +5229,11 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="57" outlineLevel="1">
       <c r="A57" s="5" t="inlineStr">
@@ -5239,7 +5243,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>未见之道</t>
+          <t>未見之道</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -5252,7 +5256,11 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr"/>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="58" outlineLevel="1">
       <c r="A58" s="5" t="inlineStr">
@@ -5262,7 +5270,7 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>无名心木</t>
+          <t>無名心木</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
@@ -5275,7 +5283,11 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="59" outlineLevel="1">
       <c r="A59" s="5" t="inlineStr">
@@ -5285,7 +5297,7 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>微小损害</t>
+          <t>微小損害</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
@@ -5298,7 +5310,11 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr"/>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="60" outlineLevel="1">
       <c r="A60" s="5" t="inlineStr">
@@ -5362,7 +5378,7 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>对你的暴击伤害加成</t>
+          <t>對你的暴擊傷害加成</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -5375,7 +5391,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr"/>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="63" outlineLevel="1">
       <c r="A63" s="5" t="inlineStr">
@@ -5385,7 +5405,7 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>图腾施放和攻击速度</t>
+          <t>圖騰攻擊及施放速度</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -5398,7 +5418,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr"/>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -5442,7 +5466,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>精算猎者</t>
+          <t>精算獵者</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -5455,7 +5479,11 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr"/>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="67" outlineLevel="1">
       <c r="A67" s="5" t="inlineStr">
@@ -5465,7 +5493,7 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>同袍情谊</t>
+          <t>同袍情誼</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
@@ -5478,7 +5506,11 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E67" s="5" t="inlineStr"/>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="68" outlineLevel="1">
       <c r="A68" s="5" t="inlineStr">
@@ -5488,7 +5520,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>暴击伤害</t>
+          <t>暴擊傷害</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -5501,7 +5533,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E68" s="5" t="inlineStr"/>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="69" outlineLevel="1">
       <c r="A69" s="5" t="inlineStr">
@@ -5511,7 +5547,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>暴击伤害</t>
+          <t>暴擊傷害</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
@@ -5524,7 +5560,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E69" s="5" t="inlineStr"/>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="70" outlineLevel="1">
       <c r="A70" s="5" t="inlineStr">
@@ -5534,7 +5574,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>暴击伤害</t>
+          <t>暴擊傷害</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
@@ -5547,7 +5587,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E70" s="5" t="inlineStr"/>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="71" outlineLevel="1">
       <c r="A71" s="5" t="inlineStr">
@@ -5557,7 +5601,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>伤害与召唤物伤害</t>
+          <t>傷害和召喚物傷害</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
@@ -5570,7 +5614,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr"/>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="72" outlineLevel="1">
       <c r="A72" s="5" t="inlineStr">
@@ -5580,7 +5628,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>伤害与召唤物伤害</t>
+          <t>傷害和召喚物傷害</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
@@ -5593,7 +5641,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E72" s="5" t="inlineStr"/>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="73" outlineLevel="1">
       <c r="A73" s="5" t="inlineStr">
@@ -5603,7 +5655,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>伤害与召唤物伤害</t>
+          <t>傷害和召喚物傷害</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -5616,12 +5668,16 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E73" s="5" t="inlineStr"/>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="74" outlineLevel="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>升华数据已与 poe2db.tw 交叉验证（2/16 条）</t>
+          <t>升华数据已与 poe2db.tw 交叉验证（16/16 条）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607160800) from my-cloud-project@86e3e15
</commit_message>
<xml_diff>
--- a/Grim_Pillars_Oracle_BD指南.xlsx
+++ b/Grim_Pillars_Oracle_BD指南.xlsx
@@ -283,7 +283,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -308,7 +308,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -333,9 +333,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -358,9 +358,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -383,9 +383,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>32</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -408,9 +408,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>37</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -433,9 +433,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>40</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -460,7 +460,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>43</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -483,12 +483,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>48</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="400050" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -510,7 +510,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -535,10 +535,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="200025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -560,10 +560,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>57</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="400050" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -583,9 +583,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>23</row>
+      <row>60</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -610,7 +610,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>63</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -633,12 +633,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>66</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="609600" cy="304800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="15" name="Image 15" descr="Picture"/>
@@ -658,9 +658,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>69</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -685,7 +685,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>32</row>
+      <row>72</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -710,7 +710,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>37</row>
+      <row>75</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -733,9 +733,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>37</row>
+      <row>88</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -760,7 +760,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>40</row>
+      <row>91</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -783,9 +783,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>40</row>
+      <row>94</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -810,7 +810,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>43</row>
+      <row>97</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -835,10 +835,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>48</row>
+      <row>100</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="400050" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="23" name="Image 23" descr="Picture"/>
@@ -860,10 +860,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>51</row>
+      <row>103</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="295275" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="24" name="Image 24" descr="Picture"/>
@@ -885,10 +885,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>54</row>
+      <row>106</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="200025" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="25" name="Image 25" descr="Picture"/>
@@ -910,10 +910,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>57</row>
+      <row>109</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="400050" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="26" name="Image 26" descr="Picture"/>
@@ -935,7 +935,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>60</row>
+      <row>112</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -946,431 +946,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId27"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>63</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="28" name="Image 28" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId28"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>66</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="304800"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="29" name="Image 29" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId29"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>69</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="30" name="Image 30" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId30"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>72</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="31" name="Image 31" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId31"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>75</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="32" name="Image 32" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId32"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>80</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="400050" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="33" name="Image 33" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId33"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>83</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="34" name="Image 34" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId34"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>88</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="35" name="Image 35" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId35"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>91</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="36" name="Image 36" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId36"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>94</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="37" name="Image 37" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId37"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>97</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="38" name="Image 38" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId38"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>100</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="39" name="Image 39" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId39"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>103</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="295275" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="40" name="Image 40" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId40"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>106</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="41" name="Image 41" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId41"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>109</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="42" name="Image 42" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId42"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>112</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="43" name="Image 43" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId43"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>115</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="44" name="Image 44" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId44"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1401,31 +976,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>105</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2577,21 +2127,18 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>法術圖騰
-(Level)
+          <t>Spell Totem
 Lv.7</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>恐怖之柱
-(Level)</t>
+          <t>Grim Pillars</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>苦澀衰亡
-(Level)</t>
+          <t>Bitter Dead</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -2608,50 +2155,25 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>達拉的渴望
-(Date)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" outlineLevel="1" ht="110" customHeight="1">
+          <t>Dialla's Desire</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" outlineLevel="1" ht="80" customHeight="1">
       <c r="A7" s="12" t="n"/>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>★ 圖騰持續時間為8秒
-★ 限制(1—2)個圖騰
-★ 圖騰獲得+(0—75)%全元素抗性
-★ 圖騰獲得+(0—35)%混沌抗性
-★ 每消耗1暴擊球插槽中的技能造成10%更多傷害
-★ 每消耗1耐力球，召喚的圖騰有20%更多生命
-★ 每消耗1耐力球，召喚的圖騰有20%更多持續時間
-★ 插槽中的法術有25%更少施放速度
-▶ 图腾施法核心</t>
+          <t>▶ 图腾施法核心</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>★ 造成(3—99)至(5—149)冰冷傷害
-★ 如果在0.5秒內被不是你的其他來源破壞，造成80%更少傷害
-★ 創造半徑為4公尺
-★ 創造8根恐怖之柱
-★ 噴發範圍為@1.2公尺
-★ 恐怖之柱持續10秒
-★ 恐怖之柱擁有(27—9536)最大生命
-★ 恐怖之柱上限為20根
-▶ BD 主伤害：铺冰柱，图腾施放免 Ward</t>
+          <t>▶ BD 主伤害：铺冰柱，图腾施放免 Ward</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>★ 轉化半徑為3.5公尺
-★ 轉化至多(1—7)具屍體
-★ 核心持續時間為5秒
-★ 造成(9—319)至(14—478)冰冷傷害
-★ 爆炸範圍為2公尺
-★ 冰緩視同對敵人造成(26—888)至(39—1332)冰冷傷害
-★ 冰緩半徑1.5公尺內的敵人
-★ 法術傷害同時影響此技能的持續傷害減益效果
-▶ 插图腾链：尸体冰霜 DoT</t>
+          <t>▶ 插图腾链：尸体冰霜 DoT</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -2668,9 +2190,7 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>★ +5%被輔助的技能的品質
-★ 被輔助的技能寶石等級+1
-▶ 达拉血统辅助</t>
+          <t>▶ 达拉血统辅助</t>
         </is>
       </c>
     </row>
@@ -2759,8 +2279,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>大法師
-(Level)
+          <t>Archmage
 Lv.21</t>
         </is>
       </c>
@@ -2776,19 +2295,15 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>阿茲里的共融
-(Date)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" outlineLevel="1" ht="84" customHeight="1">
+          <t>Atziri's Communion</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" outlineLevel="1" ht="80" customHeight="1">
       <c r="A15" s="12" t="n"/>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>★ 你每擁有100最大魔力，非引導法術獲得等同於4%傷害的額外閃電傷害
-★ 非引導法術額外消耗你最大魔力的(6.1—8)%
-★ base deal no damage 1
-▶ 法力转法术伤害</t>
+          <t>▶ 法力转法术伤害</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
@@ -2803,8 +2318,7 @@
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>★ 被輔助的技能會保留等同於66%基礎精魂保留的最大生命百分比
-▶ 插 Archmage</t>
+          <t>▶ 插 Archmage</t>
         </is>
       </c>
     </row>
@@ -2817,8 +2331,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>纏繞
-(Level)
+          <t>Entangle
 Lv.13</t>
         </is>
       </c>
@@ -2848,21 +2361,11 @@
         </is>
       </c>
     </row>
-    <row r="18" outlineLevel="1" ht="120.4" customHeight="1">
+    <row r="18" outlineLevel="1" ht="80" customHeight="1">
       <c r="A18" s="12" t="n"/>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>■ 將技能「纏結」的特效替換為獸性奔騰。
-■ 將技能「纏結」的特效替換為冥河。
-★ 造成(4—111)至(6—167)物理傷害
-★ 裂縫長度為8米
-★ 對1.5公尺內的敵人附加藤蔓
-★ 限制(4—8)道裂縫
-★ 裂縫持續時間為8秒
-★ 每0.1秒附加一條藤蔓
-★ 當過度生長時根鬚失效速度減緩25%
-★ 造成(1—29)至(1—43)物理傷害
-▶ 引爆冰柱清图</t>
+          <t>▶ 引爆冰柱清图</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -2900,8 +2403,7 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>瀆神
-(Level)
+          <t>Blasphemy
 Lv.18</t>
         </is>
       </c>
@@ -2931,20 +2433,11 @@
         </is>
       </c>
     </row>
-    <row r="21" outlineLevel="1" ht="115.2" customHeight="1">
+    <row r="21" outlineLevel="1" ht="80" customHeight="1">
       <c r="A21" s="12" t="n"/>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>■ 移除玩家極地裝甲、暴風之盾、鮮血狂怒、熔岩護盾、迷蹤、石化之血、光環、病疫之難、凋零之步、詛咒和捷光環的視覺特效。
-■ 你的光環特效替換為力場防護罩。
-■ 你的光環特效替換為一個閃耀著電光的骷髏。
-■ 你的光環特效替還為一個被地獄之火圍繞的骷髏。
-★ 插槽中的詛咒技能會以光環的形式影響周圍
-★ 每個插槽中的詛咒占用60精魂
-★ 被輔助的詛咒有(41—50)%更少效果幅度
-★ 插槽中的技能在基礎範圍上額外增加+1公尺
-★ base deal no damage 1
-▶ 诅咒光环</t>
+          <t>▶ 诅咒光环</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -2982,15 +2475,13 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>極地裝甲
-(Level)
+          <t>Arctic Armour
 Lv.19</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>極盛 II
-(Zenith II)</t>
+          <t>Zenith II</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -3009,28 +2500,16 @@
         </is>
       </c>
     </row>
-    <row r="24" outlineLevel="1" ht="120.4" customHeight="1">
+    <row r="24" outlineLevel="1" ht="80" customHeight="1">
       <c r="A24" s="12" t="n"/>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>■ 移除玩家極地裝甲、暴風之盾、鮮血狂怒、熔岩護盾、迷蹤、石化之血、光環、病疫之難、凋零之步、詛咒和捷光環的視覺特效。
-■ 將技能「極地裝甲」的特效替換為下著冰雹的雷雲。
-★ 每層造成(3—101)至(5—152)冰冷傷害
-★ 施加之冰緩具有100%更多幅度
-★ 100%更多冰凍累積
-★ 每(0.73—1.25)秒獲得1層，最多可達(2—5)層
-★ base_movement_velocity_+%
-★ mana_degeneration_per_minute
-★ physical_damage_taken_+
-★ fire_damage_taken_+
-▶ 冰霜防御</t>
+          <t>▶ 冰霜防御</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>★ 被輔助的技能增加25%魔力消耗效率
-★ 你的魔力高於最大魔力的90%時，被輔助的法術造成30%更多傷害
-▶ 零魔力技能可满层 Zenith</t>
+          <t>▶ 零魔力技能可满层 Zenith</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
@@ -3065,14 +2544,12 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>她的宣告
-(Date)</t>
+          <t>Her Declaration</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>神使之心
-(Date)</t>
+          <t>Seraph's Heart</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -3097,14 +2574,12 @@
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>★ 當被輔助的技能啟用時，進入你存在範圍內的敵人會被威嚇，持續4秒
-▶ 插 Purity of Lightning</t>
+          <t>▶ 插 Purity of Lightning</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>★ 當被輔助的技能啟用時，敵人的擊中有20%機率視你所有的抗性為90%
-▶ 插 Purity of Lightning</t>
+          <t>▶ 插 Purity of Lightning</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -3245,8 +2720,7 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>烏特雷的儀式
-(Date)</t>
+          <t>Uhtred's Rite</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
@@ -3277,10 +2751,7 @@
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>★ 被輔助的技能使用時根據每1秒冷卻時間，獲得持續1秒的滿溢聖杯
-★ 被輔助的技能在任意生命藥劑作用期間內造成20%更多傷害
-★ 被輔助的技能在任意魔力藥劑作用期間內增加20%魔力消耗效率
-▶ 插 Refutation</t>
+          <t>▶ 插 Refutation</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -3320,8 +2791,7 @@
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>卡塔爾的恢復
-(Date)</t>
+          <t>Khatal's Rejuvenation</t>
         </is>
       </c>
     </row>
@@ -3350,9 +2820,7 @@
       </c>
       <c r="E41" s="13" t="inlineStr">
         <is>
-          <t>★ 被輔助技能所創造的痕跡會在拾取時賦予卡塔爾的回春
-★ base_cooldown_speed_+%
-▶ 生命痕跡族裔辅助</t>
+          <t>▶ 生命痕跡族裔辅助</t>
         </is>
       </c>
     </row>
@@ -3791,30 +3259,17 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>林木塑像
-(Sylvan's Effigy)</t>
+          <t>Sylvan's Effigy</t>
         </is>
       </c>
       <c r="C80" s="15" t="n"/>
     </row>
-    <row r="81" outlineLevel="1" ht="264" customHeight="1">
+    <row r="81" outlineLevel="1" ht="84" customHeight="1">
       <c r="A81" s="12" t="n"/>
       <c r="B81" s="13" t="inlineStr"/>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>林木塑像 (Sylvan's Effigy)
-底材：Stoic Sceptre
-需求:  等級 62, 12 智慧
-■ 賦予技能: 紀律
-■ 賦予技能: 等級 14 阿茲莫里巨狼
-★ 增加(50—75)%精魂
-★ 處於你存在範圍中的友方每秒回復(50—100)生命
-★ +(6—12)點全部能力值
-★ 盟友對你標記的目標增加(50—100)%傷害
-★ 你可以擁有任意數量的不同類型盟友
-★ discipline art variation 1
-「Darkness howls through ancient bones, a wistful cry
-on hollow winds. The moon listens. The pack gathers.」
+          <t>Sylvan's Effigy
 ▶ BD 用途：II组主手：+58% Spirit、+6全属性，切换时保光环
 🔗 https://poe2db.tw/tw/Sylvans_Effigy
 ▶ +58% Spirit、+6 全属性，弥补 II 组无 Guiding Palm</t>
@@ -3830,27 +3285,17 @@
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>永恆火花
-(The Eternal Spark)</t>
+          <t>The Eternal Spark</t>
         </is>
       </c>
       <c r="C83" s="15" t="n"/>
     </row>
-    <row r="84" outlineLevel="1" ht="216" customHeight="1">
+    <row r="84" outlineLevel="1" ht="84" customHeight="1">
       <c r="A84" s="12" t="n"/>
       <c r="B84" s="13" t="inlineStr"/>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>永恆火花 (The Eternal Spark)
-底材：Crystal Focus
-需求:  等級 26, 38 智慧
-★ 增加(50—70)%能量護盾
-★ +5%最大閃電抗性
-★ +(20—30)%閃電抗性
-★ 增加40%魔力回復率
-★ 站立時，增加40%魔力回復率
-「A flash of blue, a stormcloud's kiss,
-her motionless dance the pulse of bliss」
+          <t>The Eternal Spark
 ▶ BD 用途：II组副手：+30%闪电抗、+5%闪电抗上限、70% ES
 🔗 https://poe2db.tw/tw/The_Eternal_Spark
 ▶ +30% 闪电抗、+5% 闪电抗上限，ES 向生存</t>
@@ -4172,21 +3617,17 @@
       </c>
       <c r="B115" s="14" t="inlineStr">
         <is>
-          <t>守護神器
-(Warding Fetish)</t>
+          <t>Warding Fetish</t>
         </is>
       </c>
       <c r="C115" s="15" t="n"/>
     </row>
-    <row r="116" outlineLevel="1" ht="108" customHeight="1">
+    <row r="116" outlineLevel="1" ht="60" customHeight="1">
       <c r="A116" s="12" t="n"/>
       <c r="B116" s="13" t="inlineStr"/>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>守護神器 (Warding Fetish)
-■ 你身上每有一個詛咒，增加30%傷害
-■ 減少30%你身上的詛咒效果
-■ 增加60%來自已裝備法器的能量護盾
+          <t>Warding Fetish
 ▶ BD 用途：涂油核心：每诅咒 +30% 伤害，-30% 诅咒效果
 🔗 https://poe2db.tw/tw/Warding_Fetish</t>
         </is>
@@ -5216,7 +4657,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>虛實交織</t>
+          <t>虚实交织</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -5229,11 +4670,7 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E56" s="5" t="inlineStr"/>
     </row>
     <row r="57" outlineLevel="1">
       <c r="A57" s="5" t="inlineStr">
@@ -5243,7 +4680,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>未見之道</t>
+          <t>未见之道</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -5256,11 +4693,7 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E57" s="5" t="inlineStr"/>
     </row>
     <row r="58" outlineLevel="1">
       <c r="A58" s="5" t="inlineStr">
@@ -5378,7 +4811,7 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>對你的暴擊傷害加成</t>
+          <t>对你的暴击伤害加成</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -5391,11 +4824,7 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E62" s="5" t="inlineStr"/>
     </row>
     <row r="63" outlineLevel="1">
       <c r="A63" s="5" t="inlineStr">
@@ -5405,7 +4834,7 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>圖騰攻擊及施放速度</t>
+          <t>图腾施放和攻击速度</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -5418,11 +4847,7 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -5466,7 +4891,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>精算獵者</t>
+          <t>精算猎者</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -5479,11 +4904,7 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E66" s="5" t="inlineStr"/>
     </row>
     <row r="67" outlineLevel="1">
       <c r="A67" s="5" t="inlineStr">
@@ -5520,7 +4941,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>暴擊傷害</t>
+          <t>暴击伤害</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -5533,11 +4954,7 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E68" s="5" t="inlineStr"/>
     </row>
     <row r="69" outlineLevel="1">
       <c r="A69" s="5" t="inlineStr">
@@ -5547,7 +4964,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>暴擊傷害</t>
+          <t>暴击伤害</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
@@ -5560,11 +4977,7 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E69" s="5" t="inlineStr"/>
     </row>
     <row r="70" outlineLevel="1">
       <c r="A70" s="5" t="inlineStr">
@@ -5574,7 +4987,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>暴擊傷害</t>
+          <t>暴击伤害</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
@@ -5587,11 +5000,7 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E70" s="5" t="inlineStr"/>
     </row>
     <row r="71" outlineLevel="1">
       <c r="A71" s="5" t="inlineStr">
@@ -5601,7 +5010,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>傷害和召喚物傷害</t>
+          <t>伤害与召唤物伤害</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
@@ -5614,11 +5023,7 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E71" s="5" t="inlineStr"/>
     </row>
     <row r="72" outlineLevel="1">
       <c r="A72" s="5" t="inlineStr">
@@ -5628,7 +5033,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>傷害和召喚物傷害</t>
+          <t>伤害与召唤物伤害</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
@@ -5641,11 +5046,7 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E72" s="5" t="inlineStr"/>
     </row>
     <row r="73" outlineLevel="1">
       <c r="A73" s="5" t="inlineStr">
@@ -5655,7 +5056,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>傷害和召喚物傷害</t>
+          <t>伤害与召唤物伤害</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -5668,16 +5069,12 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>✓poe2db</t>
-        </is>
-      </c>
+      <c r="E73" s="5" t="inlineStr"/>
     </row>
     <row r="74" outlineLevel="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>升华数据已与 poe2db.tw 交叉验证（16/16 条）</t>
+          <t>升华数据已与 poe2db.tw 交叉验证（5/16 条）</t>
         </is>
       </c>
     </row>
@@ -6219,21 +5616,17 @@
       </c>
       <c r="B105" s="14" t="inlineStr">
         <is>
-          <t>守護神器
-(Warding Fetish)</t>
+          <t>Warding Fetish</t>
         </is>
       </c>
       <c r="C105" s="15" t="n"/>
     </row>
-    <row r="106" outlineLevel="1" ht="132" customHeight="1">
+    <row r="106" outlineLevel="1" ht="84" customHeight="1">
       <c r="A106" s="12" t="n"/>
       <c r="B106" s="13" t="inlineStr"/>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>守護神器 (Warding Fetish)
-■ 你身上每有一個詛咒，增加30%傷害
-■ 減少30%你身上的詛咒效果
-■ 增加60%來自已裝備法器的能量護盾
+          <t>Warding Fetish
 ▶ BD 用途：涂油核心：每诅咒 +30% 伤害，-30% 诅咒效果
 🔗 https://poe2db.tw/tw/Warding_Fetish
 ▶ 自诅咒 → 伤害转化核心</t>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607160821) from my-cloud-project@1b8f426
</commit_message>
<xml_diff>
--- a/Grim_Pillars_Oracle_BD指南.xlsx
+++ b/Grim_Pillars_Oracle_BD指南.xlsx
@@ -283,7 +283,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -308,7 +308,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>2</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -333,9 +333,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>3</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -358,9 +358,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -383,9 +383,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>5</col>
       <colOff>0</colOff>
-      <row>32</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -408,9 +408,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>6</col>
       <colOff>0</colOff>
-      <row>37</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -433,9 +433,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>40</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -460,7 +460,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>43</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -483,12 +483,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>48</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="400050" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -510,7 +510,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>51</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -535,10 +535,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>54</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="200025" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -560,10 +560,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>57</row>
+      <row>23</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="400050" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -583,9 +583,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>60</row>
+      <row>23</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -610,7 +610,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>63</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -633,12 +633,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>66</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="304800"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="15" name="Image 15" descr="Picture"/>
@@ -658,9 +658,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>3</col>
       <colOff>0</colOff>
-      <row>69</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -685,7 +685,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>72</row>
+      <row>32</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -710,7 +710,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>75</row>
+      <row>37</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -733,9 +733,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>2</col>
       <colOff>0</colOff>
-      <row>88</row>
+      <row>37</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -760,7 +760,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>91</row>
+      <row>40</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -783,9 +783,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>4</col>
       <colOff>0</colOff>
-      <row>94</row>
+      <row>40</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -810,7 +810,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>97</row>
+      <row>43</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -835,10 +835,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>100</row>
+      <row>48</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="400050" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="23" name="Image 23" descr="Picture"/>
@@ -860,10 +860,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>103</row>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="295275" cy="609600"/>
+    <ext cx="609600" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="24" name="Image 24" descr="Picture"/>
@@ -885,10 +885,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>106</row>
+      <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="200025" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="25" name="Image 25" descr="Picture"/>
@@ -910,10 +910,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>109</row>
+      <row>57</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="609600" cy="609600"/>
+    <ext cx="400050" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="26" name="Image 26" descr="Picture"/>
@@ -935,7 +935,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>112</row>
+      <row>60</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="609600" cy="609600"/>
@@ -946,6 +946,431 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>63</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>66</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="304800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>69</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>72</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>80</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="400050" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>83</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>88</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>91</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>94</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>97</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>100</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>103</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="295275" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>106</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>109</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>112</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>115</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -976,6 +1401,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>105</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2127,18 +2577,21 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Spell Totem
+          <t>法術圖騰
+(Level)
 Lv.7</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Grim Pillars</t>
+          <t>恐怖之柱
+(Level)</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Bitter Dead</t>
+          <t>苦澀衰亡
+(Level)</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -2155,25 +2608,50 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Dialla's Desire</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" outlineLevel="1" ht="80" customHeight="1">
+          <t>達拉的渴望
+(Date)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" outlineLevel="1" ht="110" customHeight="1">
       <c r="A7" s="12" t="n"/>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>▶ 图腾施法核心</t>
+          <t>★ 圖騰持續時間為8秒
+★ 限制(1—2)個圖騰
+★ 圖騰獲得+(0—75)%全元素抗性
+★ 圖騰獲得+(0—35)%混沌抗性
+★ 每消耗1暴擊球插槽中的技能造成10%更多傷害
+★ 每消耗1耐力球，召喚的圖騰有20%更多生命
+★ 每消耗1耐力球，召喚的圖騰有20%更多持續時間
+★ 插槽中的法術有25%更少施放速度
+▶ 图腾施法核心</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>▶ BD 主伤害：铺冰柱，图腾施放免 Ward</t>
+          <t>★ 造成(3—99)至(5—149)冰冷傷害
+★ 如果在0.5秒內被不是你的其他來源破壞，造成80%更少傷害
+★ 創造半徑為4公尺
+★ 創造8根恐怖之柱
+★ 噴發範圍為@1.2公尺
+★ 恐怖之柱持續10秒
+★ 恐怖之柱擁有(27—9536)最大生命
+★ 恐怖之柱上限為20根
+▶ BD 主伤害：铺冰柱，图腾施放免 Ward</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>▶ 插图腾链：尸体冰霜 DoT</t>
+          <t>★ 轉化半徑為3.5公尺
+★ 轉化至多(1—7)具屍體
+★ 核心持續時間為5秒
+★ 造成(9—319)至(14—478)冰冷傷害
+★ 爆炸範圍為2公尺
+★ 冰緩視同對敵人造成(26—888)至(39—1332)冰冷傷害
+★ 冰緩半徑1.5公尺內的敵人
+★ 法術傷害同時影響此技能的持續傷害減益效果
+▶ 插图腾链：尸体冰霜 DoT</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -2190,7 +2668,9 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>▶ 达拉血统辅助</t>
+          <t>★ +5%被輔助的技能的品質
+★ 被輔助的技能寶石等級+1
+▶ 达拉血统辅助</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2759,8 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Archmage
+          <t>大法師
+(Level)
 Lv.21</t>
         </is>
       </c>
@@ -2295,15 +2776,19 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Atziri's Communion</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" outlineLevel="1" ht="80" customHeight="1">
+          <t>阿茲里的共融
+(Date)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" outlineLevel="1" ht="84" customHeight="1">
       <c r="A15" s="12" t="n"/>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>▶ 法力转法术伤害</t>
+          <t>★ 你每擁有100最大魔力，非引導法術獲得等同於4%傷害的額外閃電傷害
+★ 非引導法術額外消耗你最大魔力的(6.1—8)%
+★ base deal no damage 1
+▶ 法力转法术伤害</t>
         </is>
       </c>
       <c r="C15" s="13" t="inlineStr">
@@ -2318,7 +2803,8 @@
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>▶ 插 Archmage</t>
+          <t>★ 被輔助的技能會保留等同於66%基礎精魂保留的最大生命百分比
+▶ 插 Archmage</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2817,8 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Entangle
+          <t>纏繞
+(Level)
 Lv.13</t>
         </is>
       </c>
@@ -2361,11 +2848,21 @@
         </is>
       </c>
     </row>
-    <row r="18" outlineLevel="1" ht="80" customHeight="1">
+    <row r="18" outlineLevel="1" ht="120.4" customHeight="1">
       <c r="A18" s="12" t="n"/>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>▶ 引爆冰柱清图</t>
+          <t>■ 將技能「纏結」的特效替換為獸性奔騰。
+■ 將技能「纏結」的特效替換為冥河。
+★ 造成(4—111)至(6—167)物理傷害
+★ 裂縫長度為8米
+★ 對1.5公尺內的敵人附加藤蔓
+★ 限制(4—8)道裂縫
+★ 裂縫持續時間為8秒
+★ 每0.1秒附加一條藤蔓
+★ 當過度生長時根鬚失效速度減緩25%
+★ 造成(1—29)至(1—43)物理傷害
+▶ 引爆冰柱清图</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -2403,7 +2900,8 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Blasphemy
+          <t>瀆神
+(Level)
 Lv.18</t>
         </is>
       </c>
@@ -2433,11 +2931,20 @@
         </is>
       </c>
     </row>
-    <row r="21" outlineLevel="1" ht="80" customHeight="1">
+    <row r="21" outlineLevel="1" ht="115.2" customHeight="1">
       <c r="A21" s="12" t="n"/>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>▶ 诅咒光环</t>
+          <t>■ 移除玩家極地裝甲、暴風之盾、鮮血狂怒、熔岩護盾、迷蹤、石化之血、光環、病疫之難、凋零之步、詛咒和捷光環的視覺特效。
+■ 你的光環特效替換為力場防護罩。
+■ 你的光環特效替換為一個閃耀著電光的骷髏。
+■ 你的光環特效替還為一個被地獄之火圍繞的骷髏。
+★ 插槽中的詛咒技能會以光環的形式影響周圍
+★ 每個插槽中的詛咒占用60精魂
+★ 被輔助的詛咒有(41—50)%更少效果幅度
+★ 插槽中的技能在基礎範圍上額外增加+1公尺
+★ base deal no damage 1
+▶ 诅咒光环</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -2475,13 +2982,15 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Arctic Armour
+          <t>極地裝甲
+(Level)
 Lv.19</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Zenith II</t>
+          <t>極盛 II
+(Zenith II)</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -2500,16 +3009,28 @@
         </is>
       </c>
     </row>
-    <row r="24" outlineLevel="1" ht="80" customHeight="1">
+    <row r="24" outlineLevel="1" ht="120.4" customHeight="1">
       <c r="A24" s="12" t="n"/>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>▶ 冰霜防御</t>
+          <t>■ 移除玩家極地裝甲、暴風之盾、鮮血狂怒、熔岩護盾、迷蹤、石化之血、光環、病疫之難、凋零之步、詛咒和捷光環的視覺特效。
+■ 將技能「極地裝甲」的特效替換為下著冰雹的雷雲。
+★ 每層造成(3—101)至(5—152)冰冷傷害
+★ 施加之冰緩具有100%更多幅度
+★ 100%更多冰凍累積
+★ 每(0.73—1.25)秒獲得1層，最多可達(2—5)層
+★ base_movement_velocity_+%
+★ mana_degeneration_per_minute
+★ physical_damage_taken_+
+★ fire_damage_taken_+
+▶ 冰霜防御</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>▶ 零魔力技能可满层 Zenith</t>
+          <t>★ 被輔助的技能增加25%魔力消耗效率
+★ 你的魔力高於最大魔力的90%時，被輔助的法術造成30%更多傷害
+▶ 零魔力技能可满层 Zenith</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
@@ -2544,12 +3065,14 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Her Declaration</t>
+          <t>她的宣告
+(Date)</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Seraph's Heart</t>
+          <t>神使之心
+(Date)</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -2574,12 +3097,14 @@
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>▶ 插 Purity of Lightning</t>
+          <t>★ 當被輔助的技能啟用時，進入你存在範圍內的敵人會被威嚇，持續4秒
+▶ 插 Purity of Lightning</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>▶ 插 Purity of Lightning</t>
+          <t>★ 當被輔助的技能啟用時，敵人的擊中有20%機率視你所有的抗性為90%
+▶ 插 Purity of Lightning</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -2720,7 +3245,8 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Uhtred's Rite</t>
+          <t>烏特雷的儀式
+(Date)</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
@@ -2751,7 +3277,10 @@
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>▶ 插 Refutation</t>
+          <t>★ 被輔助的技能使用時根據每1秒冷卻時間，獲得持續1秒的滿溢聖杯
+★ 被輔助的技能在任意生命藥劑作用期間內造成20%更多傷害
+★ 被輔助的技能在任意魔力藥劑作用期間內增加20%魔力消耗效率
+▶ 插 Refutation</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -2791,7 +3320,8 @@
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>Khatal's Rejuvenation</t>
+          <t>卡塔爾的恢復
+(Date)</t>
         </is>
       </c>
     </row>
@@ -2820,7 +3350,9 @@
       </c>
       <c r="E41" s="13" t="inlineStr">
         <is>
-          <t>▶ 生命痕跡族裔辅助</t>
+          <t>★ 被輔助技能所創造的痕跡會在拾取時賦予卡塔爾的回春
+★ base_cooldown_speed_+%
+▶ 生命痕跡族裔辅助</t>
         </is>
       </c>
     </row>
@@ -3259,17 +3791,30 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>Sylvan's Effigy</t>
+          <t>林木塑像
+(Sylvan's Effigy)</t>
         </is>
       </c>
       <c r="C80" s="15" t="n"/>
     </row>
-    <row r="81" outlineLevel="1" ht="84" customHeight="1">
+    <row r="81" outlineLevel="1" ht="264" customHeight="1">
       <c r="A81" s="12" t="n"/>
       <c r="B81" s="13" t="inlineStr"/>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Sylvan's Effigy
+          <t>林木塑像 (Sylvan's Effigy)
+底材：Stoic Sceptre
+需求:  等級 62, 12 智慧
+■ 賦予技能: 紀律
+■ 賦予技能: 等級 14 阿茲莫里巨狼
+★ 增加(50—75)%精魂
+★ 處於你存在範圍中的友方每秒回復(50—100)生命
+★ +(6—12)點全部能力值
+★ 盟友對你標記的目標增加(50—100)%傷害
+★ 你可以擁有任意數量的不同類型盟友
+★ discipline art variation 1
+「Darkness howls through ancient bones, a wistful cry
+on hollow winds. The moon listens. The pack gathers.」
 ▶ BD 用途：II组主手：+58% Spirit、+6全属性，切换时保光环
 🔗 https://poe2db.tw/tw/Sylvans_Effigy
 ▶ +58% Spirit、+6 全属性，弥补 II 组无 Guiding Palm</t>
@@ -3285,17 +3830,27 @@
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>The Eternal Spark</t>
+          <t>永恆火花
+(The Eternal Spark)</t>
         </is>
       </c>
       <c r="C83" s="15" t="n"/>
     </row>
-    <row r="84" outlineLevel="1" ht="84" customHeight="1">
+    <row r="84" outlineLevel="1" ht="216" customHeight="1">
       <c r="A84" s="12" t="n"/>
       <c r="B84" s="13" t="inlineStr"/>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>The Eternal Spark
+          <t>永恆火花 (The Eternal Spark)
+底材：Crystal Focus
+需求:  等級 26, 38 智慧
+★ 增加(50—70)%能量護盾
+★ +5%最大閃電抗性
+★ +(20—30)%閃電抗性
+★ 增加40%魔力回復率
+★ 站立時，增加40%魔力回復率
+「A flash of blue, a stormcloud's kiss,
+her motionless dance the pulse of bliss」
 ▶ BD 用途：II组副手：+30%闪电抗、+5%闪电抗上限、70% ES
 🔗 https://poe2db.tw/tw/The_Eternal_Spark
 ▶ +30% 闪电抗、+5% 闪电抗上限，ES 向生存</t>
@@ -3617,17 +4172,21 @@
       </c>
       <c r="B115" s="14" t="inlineStr">
         <is>
-          <t>Warding Fetish</t>
+          <t>守護神器
+(Warding Fetish)</t>
         </is>
       </c>
       <c r="C115" s="15" t="n"/>
     </row>
-    <row r="116" outlineLevel="1" ht="60" customHeight="1">
+    <row r="116" outlineLevel="1" ht="108" customHeight="1">
       <c r="A116" s="12" t="n"/>
       <c r="B116" s="13" t="inlineStr"/>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>Warding Fetish
+          <t>守護神器 (Warding Fetish)
+■ 你身上每有一個詛咒，增加30%傷害
+■ 減少30%你身上的詛咒效果
+■ 增加60%來自已裝備法器的能量護盾
 ▶ BD 用途：涂油核心：每诅咒 +30% 伤害，-30% 诅咒效果
 🔗 https://poe2db.tw/tw/Warding_Fetish</t>
         </is>
@@ -4657,7 +5216,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>虚实交织</t>
+          <t>虛實交織</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -4670,7 +5229,11 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="57" outlineLevel="1">
       <c r="A57" s="5" t="inlineStr">
@@ -4680,7 +5243,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>未见之道</t>
+          <t>未見之道</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -4693,7 +5256,11 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr"/>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="58" outlineLevel="1">
       <c r="A58" s="5" t="inlineStr">
@@ -4811,7 +5378,7 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>对你的暴击伤害加成</t>
+          <t>對你的暴擊傷害加成</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -4824,7 +5391,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr"/>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="63" outlineLevel="1">
       <c r="A63" s="5" t="inlineStr">
@@ -4834,7 +5405,7 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>图腾施放和攻击速度</t>
+          <t>圖騰攻擊及施放速度</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -4847,7 +5418,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr"/>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -4891,7 +5466,7 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>精算猎者</t>
+          <t>精算獵者</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -4904,7 +5479,11 @@
           <t>升华核心</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr"/>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="67" outlineLevel="1">
       <c r="A67" s="5" t="inlineStr">
@@ -4941,7 +5520,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>暴击伤害</t>
+          <t>暴擊傷害</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -4954,7 +5533,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E68" s="5" t="inlineStr"/>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="69" outlineLevel="1">
       <c r="A69" s="5" t="inlineStr">
@@ -4964,7 +5547,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>暴击伤害</t>
+          <t>暴擊傷害</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
@@ -4977,7 +5560,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E69" s="5" t="inlineStr"/>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="70" outlineLevel="1">
       <c r="A70" s="5" t="inlineStr">
@@ -4987,7 +5574,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>暴击伤害</t>
+          <t>暴擊傷害</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
@@ -5000,7 +5587,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E70" s="5" t="inlineStr"/>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="71" outlineLevel="1">
       <c r="A71" s="5" t="inlineStr">
@@ -5010,7 +5601,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>伤害与召唤物伤害</t>
+          <t>傷害和召喚物傷害</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
@@ -5023,7 +5614,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr"/>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="72" outlineLevel="1">
       <c r="A72" s="5" t="inlineStr">
@@ -5033,7 +5628,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>伤害与召唤物伤害</t>
+          <t>傷害和召喚物傷害</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
@@ -5046,7 +5641,11 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E72" s="5" t="inlineStr"/>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="73" outlineLevel="1">
       <c r="A73" s="5" t="inlineStr">
@@ -5056,7 +5655,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>伤害与召唤物伤害</t>
+          <t>傷害和召喚物傷害</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -5069,12 +5668,16 @@
           <t>升华小点</t>
         </is>
       </c>
-      <c r="E73" s="5" t="inlineStr"/>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>✓poe2db</t>
+        </is>
+      </c>
     </row>
     <row r="74" outlineLevel="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>升华数据已与 poe2db.tw 交叉验证（5/16 条）</t>
+          <t>升华数据已与 poe2db.tw 交叉验证（16/16 条）</t>
         </is>
       </c>
     </row>
@@ -5616,17 +6219,21 @@
       </c>
       <c r="B105" s="14" t="inlineStr">
         <is>
-          <t>Warding Fetish</t>
+          <t>守護神器
+(Warding Fetish)</t>
         </is>
       </c>
       <c r="C105" s="15" t="n"/>
     </row>
-    <row r="106" outlineLevel="1" ht="84" customHeight="1">
+    <row r="106" outlineLevel="1" ht="132" customHeight="1">
       <c r="A106" s="12" t="n"/>
       <c r="B106" s="13" t="inlineStr"/>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>Warding Fetish
+          <t>守護神器 (Warding Fetish)
+■ 你身上每有一個詛咒，增加30%傷害
+■ 減少30%你身上的詛咒效果
+■ 增加60%來自已裝備法器的能量護盾
 ▶ BD 用途：涂油核心：每诅咒 +30% 伤害，-30% 诅咒效果
 🔗 https://poe2db.tw/tw/Warding_Fetish
 ▶ 自诅咒 → 伤害转化核心</t>

</xml_diff>